<commit_message>
Implemented method to distribute manure to crop areas
</commit_message>
<xml_diff>
--- a/data/prod_parameters/ManureMgmt.xlsx
+++ b/data/prod_parameters/ManureMgmt.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="870" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="847" uniqueCount="83">
   <si>
     <t>value</t>
   </si>
@@ -111,9 +111,6 @@
     <t>loss_stable</t>
   </si>
   <si>
-    <t>of total N</t>
-  </si>
-  <si>
     <t>loss_storage</t>
   </si>
   <si>
@@ -198,9 +195,6 @@
     <t>Definition mismatch? 20kg vs 30kg</t>
   </si>
   <si>
-    <t>of TAN</t>
-  </si>
-  <si>
     <t>General</t>
   </si>
   <si>
@@ -222,9 +216,6 @@
     <t>fallback OK?</t>
   </si>
   <si>
-    <t>of total N, Assume same as bulls</t>
-  </si>
-  <si>
     <t>poultry</t>
   </si>
   <si>
@@ -240,9 +231,6 @@
     <t>Assume same as laying hens for parent animals</t>
   </si>
   <si>
-    <t>of total N, assume same as laying hens for parent animals</t>
-  </si>
-  <si>
     <t>horses</t>
   </si>
   <si>
@@ -264,14 +252,29 @@
     <t>Same as cattle?? 17% is approx. avg. for cattle</t>
   </si>
   <si>
-    <t>Same as cattle?? 52% is approx. avg. for cattle</t>
+    <t>Swedish IIR 2019 Table 5-10</t>
+  </si>
+  <si>
+    <t>mammadjuren</t>
+  </si>
+  <si>
+    <t>% of total N</t>
+  </si>
+  <si>
+    <t>assume same as laying hens for parent animals</t>
+  </si>
+  <si>
+    <t>% of TAN</t>
+  </si>
+  <si>
+    <t>Assume same as solid manure</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -411,6 +414,12 @@
       <u/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -763,12 +772,13 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1090,7 +1100,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L142"/>
+  <dimension ref="A1:L145"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="14.28515625" bestFit="1" customWidth="1"/>
@@ -1106,45 +1116,45 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="B1" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="C1" s="4" t="s">
+      <c r="D1" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="E1" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G1" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="F1" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="G1" s="4" t="s">
+      <c r="H1" s="4" t="s">
         <v>40</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>41</v>
       </c>
       <c r="I1" s="4" t="s">
         <v>0</v>
       </c>
       <c r="J1" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="K1" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="L1" s="4" t="s">
         <v>43</v>
-      </c>
-      <c r="L1" s="4" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -1852,7 +1862,7 @@
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
@@ -1873,12 +1883,12 @@
         <v>22</v>
       </c>
       <c r="K31" s="1" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="E32" t="s">
         <v>25</v>
@@ -1893,12 +1903,12 @@
         <v>22</v>
       </c>
       <c r="L32" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="E33" t="s">
         <v>26</v>
@@ -1913,12 +1923,12 @@
         <v>22</v>
       </c>
       <c r="L33" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="E34" t="s">
         <v>27</v>
@@ -1933,15 +1943,15 @@
         <v>22</v>
       </c>
       <c r="L34" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B35" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E35" t="s">
         <v>20</v>
@@ -1956,7 +1966,7 @@
         <v>22</v>
       </c>
       <c r="K35" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="L35" t="s">
         <v>23</v>
@@ -1964,10 +1974,10 @@
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B36" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E36" t="s">
         <v>20</v>
@@ -1982,7 +1992,7 @@
         <v>22</v>
       </c>
       <c r="K36" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="L36" t="s">
         <v>23</v>
@@ -1990,7 +2000,7 @@
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E37" t="s">
         <v>25</v>
@@ -2005,7 +2015,7 @@
         <v>22</v>
       </c>
       <c r="K37" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L37" t="s">
         <v>23</v>
@@ -2013,10 +2023,10 @@
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
+        <v>44</v>
+      </c>
+      <c r="D38" t="s">
         <v>45</v>
-      </c>
-      <c r="D38" t="s">
-        <v>46</v>
       </c>
       <c r="E38" t="s">
         <v>25</v>
@@ -2031,7 +2041,7 @@
         <v>22</v>
       </c>
       <c r="K38" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="L38" t="s">
         <v>23</v>
@@ -2039,10 +2049,10 @@
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D39" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E39" t="s">
         <v>25</v>
@@ -2057,7 +2067,7 @@
         <v>22</v>
       </c>
       <c r="K39" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="L39" t="s">
         <v>23</v>
@@ -2065,7 +2075,7 @@
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E40" t="s">
         <v>26</v>
@@ -2080,7 +2090,7 @@
         <v>22</v>
       </c>
       <c r="K40" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L40" t="s">
         <v>23</v>
@@ -2088,10 +2098,10 @@
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
+        <v>44</v>
+      </c>
+      <c r="D41" t="s">
         <v>45</v>
-      </c>
-      <c r="D41" t="s">
-        <v>46</v>
       </c>
       <c r="E41" t="s">
         <v>26</v>
@@ -2106,7 +2116,7 @@
         <v>22</v>
       </c>
       <c r="K41" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="L41" t="s">
         <v>23</v>
@@ -2114,10 +2124,10 @@
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D42" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E42" t="s">
         <v>26</v>
@@ -2132,7 +2142,7 @@
         <v>22</v>
       </c>
       <c r="K42" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="L42" t="s">
         <v>23</v>
@@ -2140,7 +2150,7 @@
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E43" t="s">
         <v>27</v>
@@ -2155,7 +2165,7 @@
         <v>22</v>
       </c>
       <c r="K43" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L43" t="s">
         <v>23</v>
@@ -2163,10 +2173,10 @@
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
+        <v>44</v>
+      </c>
+      <c r="D44" t="s">
         <v>45</v>
-      </c>
-      <c r="D44" t="s">
-        <v>46</v>
       </c>
       <c r="E44" t="s">
         <v>27</v>
@@ -2181,7 +2191,7 @@
         <v>22</v>
       </c>
       <c r="K44" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="L44" t="s">
         <v>23</v>
@@ -2189,10 +2199,10 @@
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D45" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E45" t="s">
         <v>27</v>
@@ -2207,7 +2217,7 @@
         <v>22</v>
       </c>
       <c r="K45" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="L45" t="s">
         <v>23</v>
@@ -2215,13 +2225,13 @@
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C46" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D46" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="E46" t="s">
         <v>20</v>
@@ -2238,10 +2248,10 @@
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C47" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E47" t="s">
         <v>20</v>
@@ -2258,13 +2268,13 @@
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C48" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D48" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="E48" t="s">
         <v>25</v>
@@ -2281,10 +2291,10 @@
     </row>
     <row r="49" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C49" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E49" t="s">
         <v>25</v>
@@ -2299,18 +2309,18 @@
         <v>22</v>
       </c>
       <c r="K49" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="50" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C50" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D50" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="E50" t="s">
         <v>26</v>
@@ -2327,10 +2337,10 @@
     </row>
     <row r="51" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C51" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E51" t="s">
         <v>26</v>
@@ -2345,18 +2355,18 @@
         <v>22</v>
       </c>
       <c r="K51" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="52" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C52" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D52" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="E52" t="s">
         <v>27</v>
@@ -2373,10 +2383,10 @@
     </row>
     <row r="53" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C53" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E53" t="s">
         <v>27</v>
@@ -2391,12 +2401,12 @@
         <v>22</v>
       </c>
       <c r="K53" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="55" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B55" s="3"/>
       <c r="C55" s="3"/>
@@ -2561,7 +2571,7 @@
     </row>
     <row r="63" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="H63" t="s">
         <v>7</v>
@@ -2578,10 +2588,10 @@
     </row>
     <row r="64" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D64" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H64" t="s">
         <v>7</v>
@@ -2598,10 +2608,10 @@
     </row>
     <row r="65" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D65" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H65" t="s">
         <v>7</v>
@@ -2618,10 +2628,10 @@
     </row>
     <row r="66" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D66" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H66" t="s">
         <v>7</v>
@@ -2633,7 +2643,7 @@
         <v>8</v>
       </c>
       <c r="K66" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="L66" t="s">
         <v>12</v>
@@ -2641,10 +2651,10 @@
     </row>
     <row r="67" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D67" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H67" t="s">
         <v>7</v>
@@ -2656,7 +2666,7 @@
         <v>8</v>
       </c>
       <c r="K67" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="L67" t="s">
         <v>12</v>
@@ -2664,10 +2674,10 @@
     </row>
     <row r="68" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
+        <v>44</v>
+      </c>
+      <c r="D68" t="s">
         <v>45</v>
-      </c>
-      <c r="D68" t="s">
-        <v>46</v>
       </c>
       <c r="H68" t="s">
         <v>7</v>
@@ -2679,7 +2689,7 @@
         <v>8</v>
       </c>
       <c r="K68" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="L68" t="s">
         <v>12</v>
@@ -2687,10 +2697,10 @@
     </row>
     <row r="69" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D69" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="H69" t="s">
         <v>7</v>
@@ -2702,7 +2712,7 @@
         <v>8</v>
       </c>
       <c r="K69" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="L69" t="s">
         <v>12</v>
@@ -2710,13 +2720,13 @@
     </row>
     <row r="70" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C70" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D70" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="H70" t="s">
         <v>7</v>
@@ -2733,10 +2743,10 @@
     </row>
     <row r="71" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C71" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="H71" t="s">
         <v>7</v>
@@ -2748,7 +2758,7 @@
         <v>8</v>
       </c>
       <c r="K71" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="L71" t="s">
         <v>12</v>
@@ -2771,10 +2781,7 @@
         <v>4</v>
       </c>
       <c r="J72" t="s">
-        <v>22</v>
-      </c>
-      <c r="K72" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="L72" t="s">
         <v>23</v>
@@ -2797,10 +2804,7 @@
         <v>4</v>
       </c>
       <c r="J73" t="s">
-        <v>22</v>
-      </c>
-      <c r="K73" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="L73" t="s">
         <v>23</v>
@@ -2823,10 +2827,7 @@
         <v>20</v>
       </c>
       <c r="J74" t="s">
-        <v>22</v>
-      </c>
-      <c r="K74" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="L74" t="s">
         <v>23</v>
@@ -2834,7 +2835,7 @@
     </row>
     <row r="75" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E75" t="s">
         <v>25</v>
@@ -2849,10 +2850,7 @@
         <v>10</v>
       </c>
       <c r="J75" t="s">
-        <v>22</v>
-      </c>
-      <c r="K75" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="L75" t="s">
         <v>23</v>
@@ -2860,7 +2858,7 @@
     </row>
     <row r="76" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E76" t="s">
         <v>26</v>
@@ -2875,10 +2873,7 @@
         <v>14</v>
       </c>
       <c r="J76" t="s">
-        <v>22</v>
-      </c>
-      <c r="K76" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="L76" t="s">
         <v>23</v>
@@ -2886,7 +2881,7 @@
     </row>
     <row r="77" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E77" t="s">
         <v>27</v>
@@ -2901,10 +2896,7 @@
         <v>25</v>
       </c>
       <c r="J77" t="s">
-        <v>22</v>
-      </c>
-      <c r="K77" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="L77" t="s">
         <v>23</v>
@@ -2912,13 +2904,13 @@
     </row>
     <row r="78" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C78" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D78" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="E78" t="s">
         <v>27</v>
@@ -2933,10 +2925,7 @@
         <v>10</v>
       </c>
       <c r="J78" t="s">
-        <v>22</v>
-      </c>
-      <c r="K78" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="L78" t="s">
         <v>23</v>
@@ -2944,10 +2933,10 @@
     </row>
     <row r="79" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C79" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E79" t="s">
         <v>25</v>
@@ -2962,10 +2951,10 @@
         <v>10</v>
       </c>
       <c r="J79" t="s">
-        <v>22</v>
+        <v>79</v>
       </c>
       <c r="K79" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="L79" t="s">
         <v>23</v>
@@ -2973,10 +2962,10 @@
     </row>
     <row r="80" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C80" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E80" t="s">
         <v>26</v>
@@ -2991,10 +2980,10 @@
         <v>10</v>
       </c>
       <c r="J80" t="s">
-        <v>22</v>
+        <v>79</v>
       </c>
       <c r="K80" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="L80" t="s">
         <v>23</v>
@@ -3002,10 +2991,10 @@
     </row>
     <row r="81" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C81" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E81" t="s">
         <v>27</v>
@@ -3020,10 +3009,10 @@
         <v>35</v>
       </c>
       <c r="J81" t="s">
-        <v>22</v>
+        <v>79</v>
       </c>
       <c r="K81" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="L81" t="s">
         <v>23</v>
@@ -3031,7 +3020,7 @@
     </row>
     <row r="82" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B82" s="1"/>
       <c r="C82" s="1"/>
@@ -3050,15 +3039,15 @@
         <v>4</v>
       </c>
       <c r="J82" s="1" t="s">
-        <v>22</v>
+        <v>79</v>
       </c>
       <c r="K82" s="1" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
     </row>
     <row r="83" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B83" s="1"/>
       <c r="C83" s="1"/>
@@ -3077,15 +3066,15 @@
         <v>4</v>
       </c>
       <c r="J83" s="1" t="s">
-        <v>22</v>
+        <v>79</v>
       </c>
       <c r="K83" s="1" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
     </row>
     <row r="84" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B84" s="1"/>
       <c r="C84" s="1"/>
@@ -3104,10 +3093,10 @@
         <v>20</v>
       </c>
       <c r="J84" s="1" t="s">
-        <v>22</v>
+        <v>79</v>
       </c>
       <c r="K84" s="1" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
     </row>
     <row r="85" spans="1:12" x14ac:dyDescent="0.25">
@@ -3121,16 +3110,13 @@
         <v>28</v>
       </c>
       <c r="H85" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I85">
         <v>3</v>
       </c>
       <c r="J85" t="s">
-        <v>22</v>
-      </c>
-      <c r="K85" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="L85" t="s">
         <v>23</v>
@@ -3153,16 +3139,13 @@
         <v>28</v>
       </c>
       <c r="H86" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I86">
         <v>18</v>
       </c>
       <c r="J86" t="s">
-        <v>22</v>
-      </c>
-      <c r="K86" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="L86" t="s">
         <v>23</v>
@@ -3185,16 +3168,13 @@
         <v>28</v>
       </c>
       <c r="H87" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I87">
         <v>17</v>
       </c>
       <c r="J87" t="s">
-        <v>22</v>
-      </c>
-      <c r="K87" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="L87" t="s">
         <v>23</v>
@@ -3214,16 +3194,13 @@
         <v>28</v>
       </c>
       <c r="H88" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I88">
         <v>18</v>
       </c>
       <c r="J88" t="s">
-        <v>22</v>
-      </c>
-      <c r="K88" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="L88" t="s">
         <v>23</v>
@@ -3243,16 +3220,13 @@
         <v>28</v>
       </c>
       <c r="H89" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I89">
         <v>18</v>
       </c>
       <c r="J89" t="s">
-        <v>22</v>
-      </c>
-      <c r="K89" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="L89" t="s">
         <v>23</v>
@@ -3272,16 +3246,13 @@
         <v>28</v>
       </c>
       <c r="H90" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I90">
         <v>17</v>
       </c>
       <c r="J90" t="s">
-        <v>22</v>
-      </c>
-      <c r="K90" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="L90" t="s">
         <v>23</v>
@@ -3301,16 +3272,13 @@
         <v>28</v>
       </c>
       <c r="H91" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I91">
         <v>17</v>
       </c>
       <c r="J91" t="s">
-        <v>22</v>
-      </c>
-      <c r="K91" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="L91" t="s">
         <v>23</v>
@@ -3330,16 +3298,16 @@
         <v>28</v>
       </c>
       <c r="H92" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I92">
         <v>17</v>
       </c>
       <c r="J92" t="s">
-        <v>22</v>
+        <v>79</v>
       </c>
       <c r="K92" t="s">
-        <v>67</v>
+        <v>19</v>
       </c>
       <c r="L92" t="s">
         <v>23</v>
@@ -3356,16 +3324,13 @@
         <v>28</v>
       </c>
       <c r="H93" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I93">
         <v>30</v>
       </c>
       <c r="J93" t="s">
-        <v>22</v>
-      </c>
-      <c r="K93" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="L93" t="s">
         <v>23</v>
@@ -3373,7 +3338,7 @@
     </row>
     <row r="94" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B94" s="1"/>
       <c r="C94" s="1"/>
@@ -3386,21 +3351,21 @@
         <v>28</v>
       </c>
       <c r="H94" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I94" s="1">
         <v>3</v>
       </c>
       <c r="J94" s="1" t="s">
-        <v>22</v>
+        <v>79</v>
       </c>
       <c r="K94" s="1" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
     </row>
     <row r="95" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B95" s="1"/>
       <c r="C95" s="1"/>
@@ -3413,21 +3378,21 @@
         <v>28</v>
       </c>
       <c r="H95" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I95" s="1">
         <v>17</v>
       </c>
       <c r="J95" s="1" t="s">
-        <v>22</v>
+        <v>79</v>
       </c>
       <c r="K95" s="1" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
     </row>
     <row r="96" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A96" s="1" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B96" s="1"/>
       <c r="C96" s="1"/>
@@ -3440,21 +3405,21 @@
         <v>28</v>
       </c>
       <c r="H96" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I96" s="1">
         <v>30</v>
       </c>
       <c r="J96" s="1" t="s">
-        <v>22</v>
+        <v>79</v>
       </c>
       <c r="K96" s="1" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
     </row>
     <row r="97" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E97" t="s">
         <v>25</v>
@@ -3463,16 +3428,13 @@
         <v>28</v>
       </c>
       <c r="H97" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I97">
         <v>4</v>
       </c>
       <c r="J97" t="s">
-        <v>22</v>
-      </c>
-      <c r="K97" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="L97" t="s">
         <v>23</v>
@@ -3480,7 +3442,7 @@
     </row>
     <row r="98" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E98" t="s">
         <v>26</v>
@@ -3489,16 +3451,13 @@
         <v>28</v>
       </c>
       <c r="H98" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I98">
         <v>18</v>
       </c>
       <c r="J98" t="s">
-        <v>22</v>
-      </c>
-      <c r="K98" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="L98" t="s">
         <v>23</v>
@@ -3506,7 +3465,7 @@
     </row>
     <row r="99" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E99" t="s">
         <v>27</v>
@@ -3515,16 +3474,13 @@
         <v>28</v>
       </c>
       <c r="H99" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I99">
         <v>30</v>
       </c>
       <c r="J99" t="s">
-        <v>22</v>
-      </c>
-      <c r="K99" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="L99" t="s">
         <v>23</v>
@@ -3532,13 +3488,13 @@
     </row>
     <row r="100" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C100" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D100" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="E100" t="s">
         <v>26</v>
@@ -3547,16 +3503,13 @@
         <v>28</v>
       </c>
       <c r="H100" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I100">
         <v>5</v>
       </c>
       <c r="J100" t="s">
-        <v>22</v>
-      </c>
-      <c r="K100" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="L100" t="s">
         <v>23</v>
@@ -3564,13 +3517,13 @@
     </row>
     <row r="101" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C101" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D101" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="E101" t="s">
         <v>27</v>
@@ -3579,16 +3532,13 @@
         <v>28</v>
       </c>
       <c r="H101" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I101">
         <v>5</v>
       </c>
       <c r="J101" t="s">
-        <v>22</v>
-      </c>
-      <c r="K101" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="L101" t="s">
         <v>23</v>
@@ -3596,10 +3546,10 @@
     </row>
     <row r="102" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C102" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E102" t="s">
         <v>25</v>
@@ -3608,16 +3558,16 @@
         <v>28</v>
       </c>
       <c r="H102" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I102">
         <v>4</v>
       </c>
       <c r="J102" t="s">
-        <v>22</v>
+        <v>79</v>
       </c>
       <c r="K102" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="L102" t="s">
         <v>23</v>
@@ -3625,10 +3575,10 @@
     </row>
     <row r="103" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C103" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E103" t="s">
         <v>26</v>
@@ -3637,16 +3587,16 @@
         <v>28</v>
       </c>
       <c r="H103" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I103">
         <v>12</v>
       </c>
       <c r="J103" t="s">
-        <v>22</v>
+        <v>79</v>
       </c>
       <c r="K103" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="L103" t="s">
         <v>23</v>
@@ -3654,10 +3604,10 @@
     </row>
     <row r="104" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C104" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E104" t="s">
         <v>27</v>
@@ -3666,16 +3616,16 @@
         <v>28</v>
       </c>
       <c r="H104" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I104">
         <v>20</v>
       </c>
       <c r="J104" t="s">
-        <v>22</v>
+        <v>79</v>
       </c>
       <c r="K104" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="L104" t="s">
         <v>23</v>
@@ -3686,19 +3636,16 @@
         <v>25</v>
       </c>
       <c r="G105" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H105" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I105">
         <v>0.01</v>
       </c>
       <c r="J105" t="s">
-        <v>22</v>
-      </c>
-      <c r="K105" t="s">
-        <v>59</v>
+        <v>81</v>
       </c>
       <c r="L105" t="s">
         <v>23</v>
@@ -3709,19 +3656,16 @@
         <v>26</v>
       </c>
       <c r="G106" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H106" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I106">
         <v>1</v>
       </c>
       <c r="J106" t="s">
-        <v>22</v>
-      </c>
-      <c r="K106" t="s">
-        <v>59</v>
+        <v>81</v>
       </c>
       <c r="L106" t="s">
         <v>23</v>
@@ -3732,19 +3676,16 @@
         <v>27</v>
       </c>
       <c r="G107" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H107" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I107">
         <v>1</v>
       </c>
       <c r="J107" t="s">
-        <v>22</v>
-      </c>
-      <c r="K107" t="s">
-        <v>59</v>
+        <v>81</v>
       </c>
       <c r="L107" t="s">
         <v>23</v>
@@ -3755,19 +3696,16 @@
         <v>25</v>
       </c>
       <c r="G108" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H108" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I108">
         <v>0.5</v>
       </c>
       <c r="J108" t="s">
-        <v>22</v>
-      </c>
-      <c r="K108" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="L108" t="s">
         <v>23</v>
@@ -3778,19 +3716,16 @@
         <v>26</v>
       </c>
       <c r="G109" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H109" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I109">
         <v>0.5</v>
       </c>
       <c r="J109" t="s">
-        <v>22</v>
-      </c>
-      <c r="K109" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="L109" t="s">
         <v>23</v>
@@ -3801,19 +3736,16 @@
         <v>27</v>
       </c>
       <c r="G110" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H110" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I110">
         <v>1</v>
       </c>
       <c r="J110" t="s">
-        <v>22</v>
-      </c>
-      <c r="K110" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="L110" t="s">
         <v>23</v>
@@ -3824,19 +3756,16 @@
         <v>25</v>
       </c>
       <c r="G111" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H111" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I111">
         <v>0.3</v>
       </c>
       <c r="J111" t="s">
-        <v>22</v>
-      </c>
-      <c r="K111" t="s">
-        <v>59</v>
+        <v>81</v>
       </c>
       <c r="L111" t="s">
         <v>23</v>
@@ -3847,19 +3776,16 @@
         <v>26</v>
       </c>
       <c r="G112" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H112" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I112">
         <v>30</v>
       </c>
       <c r="J112" t="s">
-        <v>22</v>
-      </c>
-      <c r="K112" t="s">
-        <v>59</v>
+        <v>81</v>
       </c>
       <c r="L112" t="s">
         <v>23</v>
@@ -3870,19 +3796,16 @@
         <v>27</v>
       </c>
       <c r="G113" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H113" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I113">
         <v>30</v>
       </c>
       <c r="J113" t="s">
-        <v>22</v>
-      </c>
-      <c r="K113" t="s">
-        <v>59</v>
+        <v>81</v>
       </c>
       <c r="L113" t="s">
         <v>23</v>
@@ -3896,19 +3819,16 @@
         <v>25</v>
       </c>
       <c r="H114" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I114">
         <v>60</v>
       </c>
       <c r="J114" t="s">
-        <v>22</v>
-      </c>
-      <c r="K114" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="L114" t="s">
-        <v>23</v>
+        <v>77</v>
       </c>
     </row>
     <row r="115" spans="1:12" x14ac:dyDescent="0.25">
@@ -3925,19 +3845,16 @@
         <v>26</v>
       </c>
       <c r="H115" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I115">
         <v>51</v>
       </c>
       <c r="J115" t="s">
-        <v>22</v>
-      </c>
-      <c r="K115" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="L115" t="s">
-        <v>23</v>
+        <v>77</v>
       </c>
     </row>
     <row r="116" spans="1:12" x14ac:dyDescent="0.25">
@@ -3954,19 +3871,16 @@
         <v>26</v>
       </c>
       <c r="H116" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I116">
         <v>52</v>
       </c>
       <c r="J116" t="s">
-        <v>22</v>
-      </c>
-      <c r="K116" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="L116" t="s">
-        <v>23</v>
+        <v>77</v>
       </c>
     </row>
     <row r="117" spans="1:12" x14ac:dyDescent="0.25">
@@ -3980,19 +3894,16 @@
         <v>26</v>
       </c>
       <c r="H117" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I117">
         <v>51</v>
       </c>
       <c r="J117" t="s">
-        <v>22</v>
-      </c>
-      <c r="K117" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="L117" t="s">
-        <v>23</v>
+        <v>77</v>
       </c>
     </row>
     <row r="118" spans="1:12" x14ac:dyDescent="0.25">
@@ -4006,19 +3917,16 @@
         <v>26</v>
       </c>
       <c r="H118" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I118">
         <v>51</v>
       </c>
       <c r="J118" t="s">
-        <v>22</v>
-      </c>
-      <c r="K118" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="L118" t="s">
-        <v>23</v>
+        <v>77</v>
       </c>
     </row>
     <row r="119" spans="1:12" x14ac:dyDescent="0.25">
@@ -4032,19 +3940,16 @@
         <v>26</v>
       </c>
       <c r="H119" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I119">
         <v>52</v>
       </c>
       <c r="J119" t="s">
-        <v>22</v>
-      </c>
-      <c r="K119" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="L119" t="s">
-        <v>23</v>
+        <v>77</v>
       </c>
     </row>
     <row r="120" spans="1:12" x14ac:dyDescent="0.25">
@@ -4058,19 +3963,16 @@
         <v>26</v>
       </c>
       <c r="H120" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I120">
         <v>52</v>
       </c>
       <c r="J120" t="s">
-        <v>22</v>
-      </c>
-      <c r="K120" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="L120" t="s">
-        <v>23</v>
+        <v>77</v>
       </c>
     </row>
     <row r="121" spans="1:12" x14ac:dyDescent="0.25">
@@ -4084,16 +3986,16 @@
         <v>26</v>
       </c>
       <c r="H121" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I121">
         <v>52</v>
       </c>
       <c r="J121" t="s">
-        <v>22</v>
+        <v>79</v>
       </c>
       <c r="K121" t="s">
-        <v>67</v>
+        <v>19</v>
       </c>
     </row>
     <row r="122" spans="1:12" x14ac:dyDescent="0.25">
@@ -4104,342 +4006,349 @@
         <v>27</v>
       </c>
       <c r="H122" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I122">
         <v>10</v>
       </c>
       <c r="J122" t="s">
-        <v>22</v>
-      </c>
-      <c r="K122" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="L122" t="s">
-        <v>23</v>
+        <v>77</v>
       </c>
     </row>
     <row r="123" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A123" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="B123" s="1"/>
-      <c r="C123" s="1"/>
-      <c r="D123" s="1"/>
+        <v>1</v>
+      </c>
       <c r="E123" s="1" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F123" s="1"/>
       <c r="G123" s="1"/>
       <c r="H123" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I123" s="1">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="J123" s="1" t="s">
-        <v>22</v>
+        <v>79</v>
       </c>
       <c r="K123" s="1" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
     </row>
     <row r="124" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A124" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="B124" s="1"/>
-      <c r="C124" s="1"/>
-      <c r="D124" s="1"/>
-      <c r="E124" s="1" t="s">
+      <c r="A124" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="B124" s="5"/>
+      <c r="C124" s="5"/>
+      <c r="D124" s="5"/>
+      <c r="E124" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F124" s="5"/>
+      <c r="G124" s="5"/>
+      <c r="H124" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="I124" s="5">
+        <v>24</v>
+      </c>
+      <c r="J124" t="s">
+        <v>79</v>
+      </c>
+      <c r="K124" s="1"/>
+      <c r="L124" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="125" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A125" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="B125" s="5"/>
+      <c r="C125" s="5"/>
+      <c r="D125" s="5"/>
+      <c r="E125" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="F124" s="1"/>
-      <c r="G124" s="1"/>
-      <c r="H124" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="I124" s="1">
-        <v>52</v>
-      </c>
-      <c r="J124" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="K124" s="1" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="125" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A125" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="B125" s="1"/>
-      <c r="C125" s="1"/>
-      <c r="D125" s="1"/>
-      <c r="E125" s="1" t="s">
+      <c r="F125" s="5"/>
+      <c r="G125" s="5"/>
+      <c r="H125" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="I125" s="5">
+        <v>25</v>
+      </c>
+      <c r="J125" t="s">
+        <v>79</v>
+      </c>
+      <c r="K125" s="1"/>
+      <c r="L125" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="126" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A126" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="B126" s="5"/>
+      <c r="C126" s="5"/>
+      <c r="D126" s="5"/>
+      <c r="E126" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="F125" s="1"/>
-      <c r="G125" s="1"/>
-      <c r="H125" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="I125" s="1">
+      <c r="F126" s="5"/>
+      <c r="G126" s="5"/>
+      <c r="H126" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="I126" s="5">
         <v>10</v>
       </c>
-      <c r="J125" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="K125" s="1" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="126" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A126" t="s">
-        <v>68</v>
-      </c>
-      <c r="C126" t="s">
-        <v>69</v>
-      </c>
-      <c r="H126" t="s">
-        <v>35</v>
-      </c>
-      <c r="I126">
-        <v>40</v>
-      </c>
       <c r="J126" t="s">
-        <v>22</v>
-      </c>
-      <c r="K126" t="s">
-        <v>30</v>
+        <v>79</v>
+      </c>
+      <c r="K126" s="1"/>
+      <c r="L126" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="127" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A127" t="s">
-        <v>45</v>
-      </c>
-      <c r="E127" t="s">
+      <c r="A127" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B127" s="5"/>
+      <c r="C127" s="5"/>
+      <c r="D127" s="5"/>
+      <c r="E127" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F127" s="1"/>
+      <c r="G127" s="1"/>
+      <c r="H127" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="I127" s="1">
         <v>25</v>
       </c>
-      <c r="H127" t="s">
-        <v>35</v>
-      </c>
-      <c r="I127">
-        <v>70</v>
-      </c>
-      <c r="J127" t="s">
-        <v>22</v>
-      </c>
-      <c r="K127" t="s">
-        <v>30</v>
+      <c r="J127" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="K127" s="1" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="128" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>45</v>
-      </c>
-      <c r="E128" t="s">
+        <v>65</v>
+      </c>
+      <c r="C128" t="s">
+        <v>66</v>
+      </c>
+      <c r="H128" t="s">
+        <v>34</v>
+      </c>
+      <c r="I128">
+        <v>40</v>
+      </c>
+      <c r="J128" t="s">
+        <v>79</v>
+      </c>
+      <c r="L128" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="129" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A129" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B129" s="1"/>
+      <c r="C129" s="1"/>
+      <c r="D129" s="1"/>
+      <c r="E129" s="1"/>
+      <c r="F129" s="1"/>
+      <c r="G129" s="1"/>
+      <c r="H129" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="I129" s="1">
+        <v>0</v>
+      </c>
+      <c r="J129" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="K129" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="130" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A130" t="s">
+        <v>44</v>
+      </c>
+      <c r="E130" t="s">
+        <v>25</v>
+      </c>
+      <c r="H130" t="s">
+        <v>34</v>
+      </c>
+      <c r="I130">
+        <v>70</v>
+      </c>
+      <c r="J130" t="s">
+        <v>79</v>
+      </c>
+      <c r="L130" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="131" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A131" t="s">
+        <v>44</v>
+      </c>
+      <c r="E131" t="s">
         <v>26</v>
       </c>
-      <c r="H128" t="s">
-        <v>35</v>
-      </c>
-      <c r="I128">
+      <c r="H131" t="s">
+        <v>34</v>
+      </c>
+      <c r="I131">
         <v>51</v>
       </c>
-      <c r="J128" t="s">
-        <v>22</v>
-      </c>
-      <c r="K128" t="s">
+      <c r="J131" t="s">
+        <v>79</v>
+      </c>
+      <c r="L131" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="132" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A132" t="s">
+        <v>44</v>
+      </c>
+      <c r="E132" t="s">
+        <v>27</v>
+      </c>
+      <c r="H132" t="s">
+        <v>34</v>
+      </c>
+      <c r="I132">
+        <v>10</v>
+      </c>
+      <c r="J132" t="s">
+        <v>79</v>
+      </c>
+      <c r="L132" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="134" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="H134" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="I134" s="1">
+        <v>0</v>
+      </c>
+      <c r="J134" s="1"/>
+      <c r="K134" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="135" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="H135" s="1" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="129" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A129" t="s">
-        <v>45</v>
-      </c>
-      <c r="E129" t="s">
-        <v>27</v>
-      </c>
-      <c r="H129" t="s">
-        <v>35</v>
-      </c>
-      <c r="I129">
-        <v>10</v>
-      </c>
-      <c r="J129" t="s">
-        <v>22</v>
-      </c>
-      <c r="K129" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="131" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="H131" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="I131" s="1">
+      <c r="I135" s="1">
         <v>0</v>
       </c>
-      <c r="J131" s="1"/>
-      <c r="K131" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="132" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="H132" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="I132" s="1">
+      <c r="J135" s="1"/>
+      <c r="K135" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="136" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="H136" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="I136" s="1">
         <v>0</v>
       </c>
-      <c r="J132" s="1"/>
-      <c r="K132" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="133" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="H133" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="I133" s="1">
-        <v>0</v>
-      </c>
-      <c r="J133" s="1"/>
-      <c r="K133" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="134" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="H134" s="1"/>
-      <c r="I134" s="1"/>
-      <c r="J134" s="1"/>
-      <c r="K134" s="1"/>
-    </row>
-    <row r="135" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A135" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="B135" s="3"/>
-      <c r="C135" s="3"/>
-      <c r="D135" s="3"/>
-      <c r="E135" s="3"/>
-      <c r="F135" s="3"/>
-      <c r="G135" s="3"/>
-      <c r="H135" s="3"/>
-      <c r="I135" s="3"/>
-      <c r="J135" s="3"/>
-      <c r="K135" s="3"/>
-      <c r="L135" s="3"/>
-    </row>
-    <row r="136" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A136" t="s">
-        <v>1</v>
-      </c>
-      <c r="C136" t="s">
-        <v>2</v>
-      </c>
-      <c r="D136" t="s">
-        <v>3</v>
-      </c>
-      <c r="H136" t="s">
-        <v>4</v>
-      </c>
-      <c r="I136">
-        <v>5.39</v>
-      </c>
-      <c r="J136" t="s">
-        <v>5</v>
-      </c>
-      <c r="L136" t="s">
-        <v>6</v>
+      <c r="J136" s="1"/>
+      <c r="K136" s="1" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="137" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A137" t="s">
-        <v>1</v>
-      </c>
-      <c r="C137" t="s">
-        <v>9</v>
-      </c>
-      <c r="D137" t="s">
-        <v>3</v>
-      </c>
-      <c r="H137" t="s">
-        <v>4</v>
-      </c>
-      <c r="I137">
-        <v>2.8</v>
-      </c>
-      <c r="J137" t="s">
-        <v>5</v>
-      </c>
-      <c r="K137" t="s">
-        <v>10</v>
-      </c>
-      <c r="L137" t="s">
-        <v>11</v>
-      </c>
+      <c r="H137" s="1"/>
+      <c r="I137" s="1"/>
+      <c r="J137" s="1"/>
+      <c r="K137" s="1"/>
     </row>
     <row r="138" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A138" t="s">
-        <v>1</v>
-      </c>
-      <c r="D138" t="s">
-        <v>13</v>
-      </c>
-      <c r="H138" t="s">
-        <v>4</v>
-      </c>
-      <c r="I138">
-        <v>2.2599999999999998</v>
-      </c>
-      <c r="J138" t="s">
-        <v>5</v>
-      </c>
-      <c r="L138" t="s">
-        <v>11</v>
-      </c>
+      <c r="A138" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B138" s="3"/>
+      <c r="C138" s="3"/>
+      <c r="D138" s="3"/>
+      <c r="E138" s="3"/>
+      <c r="F138" s="3"/>
+      <c r="G138" s="3"/>
+      <c r="H138" s="3"/>
+      <c r="I138" s="3"/>
+      <c r="J138" s="3"/>
+      <c r="K138" s="3"/>
+      <c r="L138" s="3"/>
     </row>
     <row r="139" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>1</v>
       </c>
+      <c r="C139" t="s">
+        <v>2</v>
+      </c>
       <c r="D139" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="H139" t="s">
         <v>4</v>
       </c>
       <c r="I139">
-        <v>0.79</v>
+        <v>5.39</v>
       </c>
       <c r="J139" t="s">
         <v>5</v>
       </c>
-      <c r="K139" t="s">
-        <v>15</v>
-      </c>
       <c r="L139" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="140" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>1</v>
       </c>
+      <c r="C140" t="s">
+        <v>9</v>
+      </c>
       <c r="D140" t="s">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="H140" t="s">
         <v>4</v>
       </c>
       <c r="I140">
-        <v>2.2599999999999998</v>
+        <v>2.8</v>
       </c>
       <c r="J140" t="s">
         <v>5</v>
       </c>
+      <c r="K140" t="s">
+        <v>10</v>
+      </c>
       <c r="L140" t="s">
         <v>11</v>
       </c>
@@ -4449,7 +4358,7 @@
         <v>1</v>
       </c>
       <c r="D141" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="H141" t="s">
         <v>4</v>
@@ -4469,18 +4378,81 @@
         <v>1</v>
       </c>
       <c r="D142" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="H142" t="s">
         <v>4</v>
       </c>
       <c r="I142">
-        <v>2.2599999999999998</v>
+        <v>0.79</v>
       </c>
       <c r="J142" t="s">
         <v>5</v>
       </c>
       <c r="K142" t="s">
+        <v>15</v>
+      </c>
+      <c r="L142" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="143" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A143" t="s">
+        <v>1</v>
+      </c>
+      <c r="D143" t="s">
+        <v>17</v>
+      </c>
+      <c r="H143" t="s">
+        <v>4</v>
+      </c>
+      <c r="I143">
+        <v>2.2599999999999998</v>
+      </c>
+      <c r="J143" t="s">
+        <v>5</v>
+      </c>
+      <c r="L143" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="144" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A144" t="s">
+        <v>1</v>
+      </c>
+      <c r="D144" t="s">
+        <v>16</v>
+      </c>
+      <c r="H144" t="s">
+        <v>4</v>
+      </c>
+      <c r="I144">
+        <v>2.2599999999999998</v>
+      </c>
+      <c r="J144" t="s">
+        <v>5</v>
+      </c>
+      <c r="L144" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="145" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A145" t="s">
+        <v>1</v>
+      </c>
+      <c r="D145" t="s">
+        <v>18</v>
+      </c>
+      <c r="H145" t="s">
+        <v>4</v>
+      </c>
+      <c r="I145">
+        <v>2.2599999999999998</v>
+      </c>
+      <c r="J145" t="s">
+        <v>5</v>
+      </c>
+      <c r="K145" t="s">
         <v>19</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Implemented soil N2O calculations
</commit_message>
<xml_diff>
--- a/data/prod_parameters/ManureMgmt.xlsx
+++ b/data/prod_parameters/ManureMgmt.xlsx
@@ -267,7 +267,7 @@
     <t>% of TAN</t>
   </si>
   <si>
-    <t>Assume same as solid manure</t>
+    <t>Table 3.9. EMEP/EEA air pollutant emission inventory Guidebook 2019</t>
   </si>
 </sst>
 </file>
@@ -4022,21 +4022,22 @@
       <c r="A123" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E123" s="1" t="s">
+      <c r="E123" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="F123" s="1"/>
-      <c r="G123" s="1"/>
-      <c r="H123" s="1" t="s">
+      <c r="F123" s="5"/>
+      <c r="G123" s="5"/>
+      <c r="H123" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="I123" s="1">
-        <v>52</v>
-      </c>
-      <c r="J123" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="K123" s="1" t="s">
+      <c r="I123" s="5">
+        <v>60</v>
+      </c>
+      <c r="J123" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="K123" s="1"/>
+      <c r="L123" t="s">
         <v>82</v>
       </c>
     </row>
@@ -4119,27 +4120,28 @@
       </c>
     </row>
     <row r="127" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A127" s="1" t="s">
+      <c r="A127" s="5" t="s">
         <v>70</v>
       </c>
       <c r="B127" s="5"/>
       <c r="C127" s="5"/>
       <c r="D127" s="5"/>
-      <c r="E127" s="1" t="s">
+      <c r="E127" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="F127" s="1"/>
-      <c r="G127" s="1"/>
-      <c r="H127" s="1" t="s">
+      <c r="F127" s="5"/>
+      <c r="G127" s="5"/>
+      <c r="H127" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="I127" s="1">
-        <v>25</v>
-      </c>
-      <c r="J127" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="K127" s="1" t="s">
+      <c r="I127" s="5">
+        <v>60</v>
+      </c>
+      <c r="J127" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="K127" s="1"/>
+      <c r="L127" t="s">
         <v>82</v>
       </c>
     </row>

</xml_diff>